<commit_message>
Update MOF database to V2.0.0 from Revision F
</commit_message>
<xml_diff>
--- a/88MOFs_UFF_UMLIP_DATABASE_V2.0.0.xlsx
+++ b/88MOFs_UFF_UMLIP_DATABASE_V2.0.0.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sbonakala\Desktop\MATLANTIS_WORK\FRESH_SCREENING_WITH_RECENT_CSD_DATABASE\Manuscript\SUBMISSION_VERSION\Chem_Sci\comments\Rev_F\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FE7F5257-E0F7-4A1A-972D-65686F3A351D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0DC7F2F3-6898-4806-9EF0-F6845E97BF3A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="518" uniqueCount="319">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="519" uniqueCount="320">
   <si>
     <t>NOPGUY_P1</t>
   </si>
@@ -1030,6 +1030,9 @@
   </si>
   <si>
     <t>bulk_modulus_B0_GPa</t>
+  </si>
+  <si>
+    <t>NA</t>
   </si>
 </sst>
 </file>
@@ -1121,7 +1124,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1135,6 +1138,9 @@
     <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="11" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -3377,7 +3383,7 @@
         <v>4.0244716436482069</v>
       </c>
       <c r="AF20">
-        <v>1.9805999999999999</v>
+        <v>3.7574000000000001</v>
       </c>
     </row>
     <row r="21" spans="1:32" x14ac:dyDescent="0.35">
@@ -9220,8 +9226,8 @@
         <f t="shared" si="11"/>
         <v>20.938422962462312</v>
       </c>
-      <c r="AF80">
-        <v>33.079000000000001</v>
+      <c r="AF80" s="9" t="s">
+        <v>319</v>
       </c>
     </row>
     <row r="81" spans="1:32" x14ac:dyDescent="0.35">

</xml_diff>